<commit_message>
added monthly tone with and without retweets
</commit_message>
<xml_diff>
--- a/notebooks/1_temporal/tone_frequencies+retweets.xlsx
+++ b/notebooks/1_temporal/tone_frequencies+retweets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olddominion-my.sharepoint.com/personal/jmart130_odu_edu/Documents/GITHUB_VMASC/twitter_analysis_col/notebooks/1_temporal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="531" documentId="11_4C1CE49650B0F515CA3E72BFC370B3F462223BE8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB824696-A682-C846-AF9F-5387DED14154}"/>
+  <xr:revisionPtr revIDLastSave="550" documentId="11_4C1CE49650B0F515CA3E72BFC370B3F462223BE8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0986C266-55C4-EF47-BEA8-E33319B5C738}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{61C9C911-FF89-4C19-BE5A-DC4DFBA47279}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{61C9C911-FF89-4C19-BE5A-DC4DFBA47279}"/>
   </bookViews>
   <sheets>
     <sheet name="yearly" sheetId="11" r:id="rId1"/>
@@ -538,7 +538,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -571,7 +571,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -30745,15 +30744,15 @@
         <f t="shared" ref="L2:L10" si="0">$M$11</f>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M2" s="16">
+      <c r="M2" s="4">
         <f t="shared" ref="M2:M10" si="1">I2/SUM($I2:$K2)</f>
         <v>0.48067750413705829</v>
       </c>
-      <c r="N2" s="16">
+      <c r="N2" s="4">
         <f t="shared" ref="N2:N10" si="2">J2/SUM($I2:$K2)</f>
         <v>0.31626593984230505</v>
       </c>
-      <c r="O2" s="16">
+      <c r="O2" s="4">
         <f t="shared" ref="O2:O10" si="3">K2/SUM($I2:$K2)</f>
         <v>0.20305655602063663</v>
       </c>
@@ -30798,15 +30797,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M3" s="16">
+      <c r="M3" s="4">
         <f t="shared" si="1"/>
         <v>0.56864375942194734</v>
       </c>
-      <c r="N3" s="16">
+      <c r="N3" s="4">
         <f t="shared" si="2"/>
         <v>0.24738784633778654</v>
       </c>
-      <c r="O3" s="16">
+      <c r="O3" s="4">
         <f t="shared" si="3"/>
         <v>0.18396839424026615</v>
       </c>
@@ -30851,15 +30850,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M4" s="16">
+      <c r="M4" s="4">
         <f t="shared" si="1"/>
         <v>0.42147368421052633</v>
       </c>
-      <c r="N4" s="16">
+      <c r="N4" s="4">
         <f t="shared" si="2"/>
         <v>0.36643609022556389</v>
       </c>
-      <c r="O4" s="16">
+      <c r="O4" s="4">
         <f t="shared" si="3"/>
         <v>0.21209022556390977</v>
       </c>
@@ -30904,15 +30903,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M5" s="16">
+      <c r="M5" s="4">
         <f t="shared" si="1"/>
         <v>0.43021560254140195</v>
       </c>
-      <c r="N5" s="16">
+      <c r="N5" s="4">
         <f t="shared" si="2"/>
         <v>0.36987466583342016</v>
       </c>
-      <c r="O5" s="16">
+      <c r="O5" s="4">
         <f t="shared" si="3"/>
         <v>0.19990973162517794</v>
       </c>
@@ -30957,15 +30956,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M6" s="16">
+      <c r="M6" s="4">
         <f t="shared" si="1"/>
         <v>0.31206346097345999</v>
       </c>
-      <c r="N6" s="16">
+      <c r="N6" s="4">
         <f t="shared" si="2"/>
         <v>0.47457447850357459</v>
       </c>
-      <c r="O6" s="16">
+      <c r="O6" s="4">
         <f t="shared" si="3"/>
         <v>0.21336206052296544</v>
       </c>
@@ -31010,15 +31009,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="4">
         <f t="shared" si="1"/>
         <v>0.41544129295768967</v>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="4">
         <f t="shared" si="2"/>
         <v>0.35914371221264324</v>
       </c>
-      <c r="O7" s="16">
+      <c r="O7" s="4">
         <f t="shared" si="3"/>
         <v>0.22541499482966706</v>
       </c>
@@ -31063,15 +31062,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M8" s="16">
+      <c r="M8" s="4">
         <f t="shared" si="1"/>
         <v>0.43185469769853246</v>
       </c>
-      <c r="N8" s="16">
+      <c r="N8" s="4">
         <f t="shared" si="2"/>
         <v>0.33952454434072771</v>
       </c>
-      <c r="O8" s="16">
+      <c r="O8" s="4">
         <f t="shared" si="3"/>
         <v>0.22862075796073983</v>
       </c>
@@ -31116,15 +31115,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M9" s="16">
+      <c r="M9" s="4">
         <f t="shared" si="1"/>
         <v>0.41631795282226325</v>
       </c>
-      <c r="N9" s="16">
+      <c r="N9" s="4">
         <f t="shared" si="2"/>
         <v>0.32734755750134492</v>
       </c>
-      <c r="O9" s="16">
+      <c r="O9" s="4">
         <f t="shared" si="3"/>
         <v>0.25633448967639177</v>
       </c>
@@ -31169,15 +31168,15 @@
         <f t="shared" si="0"/>
         <v>0.43795899518883746</v>
       </c>
-      <c r="M10" s="16">
+      <c r="M10" s="4">
         <f t="shared" si="1"/>
         <v>0.4649430019366585</v>
       </c>
-      <c r="N10" s="16">
+      <c r="N10" s="4">
         <f t="shared" si="2"/>
         <v>0.33352274703992763</v>
       </c>
-      <c r="O10" s="16">
+      <c r="O10" s="4">
         <f t="shared" si="3"/>
         <v>0.20153425102341385</v>
       </c>

</xml_diff>